<commit_message>
feat: implement admin order entry and collection management features
</commit_message>
<xml_diff>
--- a/client/public/ALL unimported invoices.xlsx
+++ b/client/public/ALL unimported invoices.xlsx
@@ -19,10 +19,10 @@
     <sheet name="POLICE NOT FOUND" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DINOSHAN!$A$1:$E$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DINOSHAN!$A$1:$E$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'POLICE NOT FOUND'!$A$1:$G$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">RATHAN!$A$1:$E$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">ROHILAN!$A$1:$E$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">RATHAN!$A$1:$E$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">ROHILAN!$A$1:$E$40</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1276,7 +1276,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{43268C50-0890-4D3F-B29B-A18ECB921191}">
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.140625" bestFit="1" customWidth="1"/>
@@ -1339,686 +1339,295 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B4" s="7">
-        <v>46231</v>
+        <v>46223</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D4" s="5">
-        <v>6696</v>
+        <v>36364</v>
       </c>
       <c r="E4">
-        <v>25</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B5" s="7">
-        <v>46223</v>
+        <v>46127</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D5" s="5">
-        <v>36364</v>
+        <v>2252</v>
       </c>
       <c r="E5">
-        <v>33</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B6" s="7">
-        <v>46135</v>
+        <v>45527</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D6" s="5">
-        <v>400</v>
+        <v>47723</v>
       </c>
       <c r="E6">
-        <v>121</v>
+        <v>729</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B7" s="7">
-        <v>46190</v>
+        <v>45545</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D7" s="5">
-        <v>20655</v>
+        <v>128401</v>
       </c>
       <c r="E7">
-        <v>66</v>
+        <v>711</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B8" s="7">
-        <v>46248</v>
+        <v>45643</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="D8" s="5">
-        <v>23833</v>
+        <v>11040</v>
       </c>
       <c r="E8">
-        <v>8</v>
+        <v>613</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="B9" s="7">
-        <v>46127</v>
+        <v>46169</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="D9" s="5">
-        <v>2252</v>
+        <v>8748</v>
       </c>
       <c r="E9">
-        <v>129</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B10" s="7">
-        <v>45527</v>
+        <v>46184</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="D10" s="5">
-        <v>47723</v>
+        <v>11892</v>
       </c>
       <c r="E10">
-        <v>729</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="B11" s="7">
-        <v>45545</v>
+        <v>46241</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="D11" s="5">
-        <v>128401</v>
+        <v>1785</v>
       </c>
       <c r="E11">
-        <v>711</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="B12" s="7">
-        <v>45643</v>
+        <v>46212</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="D12" s="5">
-        <v>11040</v>
+        <v>8</v>
       </c>
       <c r="E12">
-        <v>613</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="B13" s="7">
-        <v>46238</v>
+        <v>46245</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="D13" s="5">
-        <v>12528</v>
+        <v>83880</v>
       </c>
       <c r="E13">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="B14" s="7">
-        <v>46154</v>
+        <v>46255</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D14" s="5">
-        <v>6003</v>
+        <v>40260</v>
       </c>
       <c r="E14">
-        <v>102</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="B15" s="7">
-        <v>46224</v>
+        <v>46254</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="D15" s="5">
-        <v>10000</v>
+        <v>43020</v>
       </c>
       <c r="E15">
-        <v>32</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="B16" s="7">
-        <v>46237</v>
+        <v>46242</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="D16" s="5">
-        <v>64400</v>
+        <v>8433</v>
       </c>
       <c r="E16">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="B17" s="7">
-        <v>46250</v>
+        <v>46254</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D17" s="5">
-        <v>30120</v>
+        <v>34614</v>
       </c>
       <c r="E17">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
       <c r="B18" s="7">
-        <v>45906</v>
+        <v>46210</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>30</v>
+        <v>53</v>
       </c>
       <c r="D18" s="5">
-        <v>4536</v>
+        <v>6480</v>
       </c>
       <c r="E18">
-        <v>350</v>
+        <v>46</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="B19" s="7">
-        <v>45531</v>
+        <v>46147</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D19" s="5">
-        <v>31140</v>
+        <v>1785</v>
       </c>
       <c r="E19">
-        <v>725</v>
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>33</v>
+        <v>61</v>
       </c>
       <c r="B20" s="7">
-        <v>46169</v>
+        <v>46251</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>34</v>
+        <v>62</v>
       </c>
       <c r="D20" s="5">
-        <v>8748</v>
+        <v>13844</v>
       </c>
       <c r="E20">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>33</v>
-      </c>
-      <c r="B21" s="7">
-        <v>46184</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D21" s="5">
-        <v>11892</v>
-      </c>
-      <c r="E21">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="7">
-        <v>46241</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D22" s="5">
-        <v>1785</v>
-      </c>
-      <c r="E22">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>37</v>
-      </c>
-      <c r="B23" s="7">
-        <v>46212</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="D23" s="5">
-        <v>8</v>
-      </c>
-      <c r="E23">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24" s="7">
-        <v>46245</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D24" s="5">
-        <v>83880</v>
-      </c>
-      <c r="E24">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>37</v>
-      </c>
-      <c r="B25" s="7">
-        <v>46255</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="D25" s="5">
-        <v>40260</v>
-      </c>
-      <c r="E25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>41</v>
-      </c>
-      <c r="B26" s="7">
-        <v>46254</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D26" s="5">
-        <v>43020</v>
-      </c>
-      <c r="E26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>43</v>
-      </c>
-      <c r="B27" s="7">
-        <v>46191</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" s="5">
-        <v>22464</v>
-      </c>
-      <c r="E27">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>45</v>
-      </c>
-      <c r="B28" s="7">
-        <v>46242</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D28" s="5">
-        <v>8433</v>
-      </c>
-      <c r="E28">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>47</v>
-      </c>
-      <c r="B29" s="7">
-        <v>46254</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D29" s="5">
-        <v>34614</v>
-      </c>
-      <c r="E29">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>49</v>
-      </c>
-      <c r="B30" s="7">
-        <v>46164</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="D30" s="5">
-        <v>13000</v>
-      </c>
-      <c r="E30">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31" s="7">
-        <v>46213</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" s="5">
-        <v>49011</v>
-      </c>
-      <c r="E31">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>52</v>
-      </c>
-      <c r="B32" s="7">
-        <v>46210</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D32" s="5">
-        <v>6480</v>
-      </c>
-      <c r="E32">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>54</v>
-      </c>
-      <c r="B33" s="7">
-        <v>46147</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D33" s="5">
-        <v>1785</v>
-      </c>
-      <c r="E33">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>56</v>
-      </c>
-      <c r="B34" s="7">
-        <v>46043</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D34" s="5">
-        <v>9682</v>
-      </c>
-      <c r="E34">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>58</v>
-      </c>
-      <c r="B35" s="7">
-        <v>46226</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D35" s="5">
-        <v>30000</v>
-      </c>
-      <c r="E35">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="7">
-        <v>46252</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="D36" s="5">
-        <v>97107</v>
-      </c>
-      <c r="E36">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>61</v>
-      </c>
-      <c r="B37" s="7">
-        <v>46251</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D37" s="5">
-        <v>13844</v>
-      </c>
-      <c r="E37">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>63</v>
-      </c>
-      <c r="B38" s="7">
-        <v>46238</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D38" s="5">
-        <v>17042</v>
-      </c>
-      <c r="E38">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" s="7">
-        <v>46247</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="D39" s="5">
-        <v>21081</v>
-      </c>
-      <c r="E39">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>66</v>
-      </c>
-      <c r="B40" s="7">
-        <v>46213</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D40" s="5">
-        <v>3024</v>
-      </c>
-      <c r="E40">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>66</v>
-      </c>
-      <c r="B41" s="7">
-        <v>46238</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D41" s="5">
-        <v>15696</v>
-      </c>
-      <c r="E41">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>69</v>
-      </c>
-      <c r="B42" s="7">
-        <v>46231</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D42" s="5">
-        <v>9904</v>
-      </c>
-      <c r="E42">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>69</v>
-      </c>
-      <c r="B43" s="7">
-        <v>46244</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D43" s="5">
-        <v>21031</v>
-      </c>
-      <c r="E43">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E43" xr:uid="{43268C50-0890-4D3F-B29B-A18ECB921191}"/>
+  <autoFilter ref="A1:E20" xr:uid="{43268C50-0890-4D3F-B29B-A18ECB921191}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2026,7 +1635,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D35D26C-6FD3-43A4-A5FF-70AAE5C4E6B6}">
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.140625" bestFit="1" customWidth="1"/>
@@ -2089,608 +1698,404 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B4" s="7">
-        <v>46142</v>
+        <v>46245</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D4" s="5">
-        <v>22148</v>
+        <v>66644</v>
       </c>
       <c r="E4">
-        <v>114</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B5" s="7">
-        <v>46245</v>
+        <v>46235</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D5" s="5">
-        <v>301637</v>
+        <v>4216</v>
       </c>
       <c r="E5">
-        <v>11</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="B6" s="7">
-        <v>46245</v>
+        <v>45951</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D6" s="5">
-        <v>66644</v>
+        <v>6</v>
       </c>
       <c r="E6">
-        <v>11</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B7" s="7">
-        <v>46235</v>
+        <v>46250</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D7" s="5">
-        <v>4216</v>
+        <v>9672</v>
       </c>
       <c r="E7">
-        <v>21</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="B8" s="7">
-        <v>46107</v>
+        <v>45903</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="D8" s="5">
-        <v>1096</v>
+        <v>1428</v>
       </c>
       <c r="E8">
-        <v>149</v>
+        <v>353</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="B9" s="7">
-        <v>46237</v>
+        <v>46245</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D9" s="5">
-        <v>6048</v>
+        <v>91044</v>
       </c>
       <c r="E9">
-        <v>19</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="B10" s="7">
-        <v>46237</v>
+        <v>46250</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="D10" s="5">
-        <v>6322</v>
+        <v>34596</v>
       </c>
       <c r="E10">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="B11" s="7">
-        <v>46244</v>
+        <v>46107</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="D11" s="5">
-        <v>40320</v>
+        <v>5000</v>
       </c>
       <c r="E11">
-        <v>12</v>
+        <v>149</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="B12" s="7">
-        <v>45951</v>
+        <v>46255</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="D12" s="5">
-        <v>6</v>
+        <v>29445</v>
       </c>
       <c r="E12">
-        <v>305</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="B13" s="7">
-        <v>46250</v>
+        <v>46196</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D13" s="5">
-        <v>9672</v>
+        <v>16004</v>
       </c>
       <c r="E13">
-        <v>6</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="B14" s="7">
-        <v>45903</v>
+        <v>46221</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
       <c r="D14" s="5">
-        <v>1428</v>
+        <v>55930</v>
       </c>
       <c r="E14">
-        <v>353</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="B15" s="7">
-        <v>46245</v>
+        <v>46231</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D15" s="5">
-        <v>91044</v>
+        <v>78624</v>
       </c>
       <c r="E15">
-        <v>11</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>94</v>
+        <v>106</v>
       </c>
       <c r="B16" s="7">
-        <v>46250</v>
+        <v>46244</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="D16" s="5">
-        <v>34596</v>
+        <v>49794</v>
       </c>
       <c r="E16">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B17" s="7">
-        <v>46107</v>
+        <v>46250</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="D17" s="5">
-        <v>5000</v>
+        <v>33513</v>
       </c>
       <c r="E17">
-        <v>149</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="B18" s="7">
-        <v>46255</v>
+        <v>46151</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="D18" s="5">
-        <v>29445</v>
+        <v>458</v>
       </c>
       <c r="E18">
-        <v>1</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="B19" s="7">
-        <v>46244</v>
+        <v>46240</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>101</v>
+        <v>115</v>
       </c>
       <c r="D19" s="5">
-        <v>4968</v>
+        <v>7142</v>
       </c>
       <c r="E19">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B20" s="7">
-        <v>46196</v>
+        <v>46251</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D20" s="5">
-        <v>16004</v>
+        <v>10713</v>
       </c>
       <c r="E20">
-        <v>60</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B21" s="7">
-        <v>45726</v>
+        <v>45975</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="D21" s="5">
-        <v>16200</v>
+        <v>4726</v>
       </c>
       <c r="E21">
-        <v>530</v>
+        <v>281</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="B22" s="7">
-        <v>46221</v>
+        <v>46226</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="D22" s="5">
-        <v>55930</v>
+        <v>35571</v>
       </c>
       <c r="E22">
-        <v>35</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B23" s="7">
-        <v>46231</v>
+        <v>46149</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="D23" s="5">
-        <v>78624</v>
+        <v>54</v>
       </c>
       <c r="E23">
-        <v>25</v>
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>106</v>
+        <v>121</v>
       </c>
       <c r="B24" s="7">
-        <v>46244</v>
+        <v>46227</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="D24" s="5">
-        <v>49794</v>
+        <v>4216</v>
       </c>
       <c r="E24">
-        <v>12</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>110</v>
+        <v>129</v>
       </c>
       <c r="B25" s="7">
-        <v>46250</v>
+        <v>46231</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>111</v>
+        <v>130</v>
       </c>
       <c r="D25" s="5">
-        <v>33513</v>
+        <v>36007</v>
       </c>
       <c r="E25">
-        <v>6</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>112</v>
+        <v>133</v>
       </c>
       <c r="B26" s="7">
-        <v>46151</v>
+        <v>46227</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>113</v>
+        <v>134</v>
       </c>
       <c r="D26" s="5">
-        <v>458</v>
+        <v>4216</v>
       </c>
       <c r="E26">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>114</v>
-      </c>
-      <c r="B27" s="7">
-        <v>46240</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D27" s="5">
-        <v>7142</v>
-      </c>
-      <c r="E27">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>114</v>
-      </c>
-      <c r="B28" s="7">
-        <v>46251</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="D28" s="5">
-        <v>10713</v>
-      </c>
-      <c r="E28">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>117</v>
-      </c>
-      <c r="B29" s="7">
-        <v>45975</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D29" s="5">
-        <v>4726</v>
-      </c>
-      <c r="E29">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>119</v>
-      </c>
-      <c r="B30" s="7">
-        <v>46226</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="D30" s="5">
-        <v>35571</v>
-      </c>
-      <c r="E30">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>121</v>
-      </c>
-      <c r="B31" s="7">
-        <v>46149</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="D31" s="5">
-        <v>54</v>
-      </c>
-      <c r="E31">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>121</v>
-      </c>
-      <c r="B32" s="7">
-        <v>46227</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D32" s="5">
-        <v>4216</v>
-      </c>
-      <c r="E32">
         <v>29</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>124</v>
-      </c>
-      <c r="B33" s="7">
-        <v>46228</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D33" s="5">
-        <v>1620</v>
-      </c>
-      <c r="E33">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>124</v>
-      </c>
-      <c r="B34" s="7">
-        <v>46230</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D34" s="5">
-        <v>7</v>
-      </c>
-      <c r="E34">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>127</v>
-      </c>
-      <c r="B35" s="7">
-        <v>45259</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D35" s="5">
-        <v>6330</v>
-      </c>
-      <c r="E35">
-        <v>997</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>129</v>
-      </c>
-      <c r="B36" s="7">
-        <v>46231</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="D36" s="5">
-        <v>36007</v>
-      </c>
-      <c r="E36">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>131</v>
-      </c>
-      <c r="B37" s="7">
-        <v>45530</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="D37" s="5">
-        <v>15639</v>
-      </c>
-      <c r="E37">
-        <v>726</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>133</v>
-      </c>
-      <c r="B38" s="7">
-        <v>46227</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="D38" s="5">
-        <v>4216</v>
-      </c>
-      <c r="E38">
-        <v>29</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E38" xr:uid="{9D35D26C-6FD3-43A4-A5FF-70AAE5C4E6B6}"/>
+  <autoFilter ref="A1:E26" xr:uid="{9D35D26C-6FD3-43A4-A5FF-70AAE5C4E6B6}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7ECFBB88-5200-475D-B171-1F2F42D2B185}">
-  <dimension ref="A1:E69"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.5703125" customWidth="1"/>
@@ -2957,931 +2362,387 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="B16" s="7">
-        <v>45768</v>
+        <v>46244</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="D16" s="5">
-        <v>1000</v>
+        <v>28147</v>
       </c>
       <c r="E16">
-        <v>488</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B17" s="7">
-        <v>45859</v>
+        <v>46174</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D17" s="5">
-        <v>242</v>
+        <v>16865</v>
       </c>
       <c r="E17">
-        <v>397</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B18" s="7">
-        <v>46181</v>
+        <v>46146</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D18" s="5">
-        <v>11001</v>
+        <v>435</v>
       </c>
       <c r="E18">
-        <v>75</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="B19" s="7">
-        <v>46235</v>
+        <v>46185</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="D19" s="5">
-        <v>11040</v>
+        <v>10844</v>
       </c>
       <c r="E19">
-        <v>21</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B20" s="7">
-        <v>46244</v>
+        <v>46250</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D20" s="5">
-        <v>28147</v>
+        <v>14764</v>
       </c>
       <c r="E20">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="B21" s="7">
-        <v>46174</v>
+        <v>46093</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="D21" s="5">
-        <v>16865</v>
+        <v>9432</v>
       </c>
       <c r="E21">
-        <v>82</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="B22" s="7">
-        <v>46146</v>
+        <v>46162</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="D22" s="5">
-        <v>435</v>
+        <v>10044</v>
       </c>
       <c r="E22">
-        <v>110</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B23" s="7">
-        <v>46185</v>
+        <v>46225</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="D23" s="5">
-        <v>10844</v>
+        <v>29612</v>
       </c>
       <c r="E23">
-        <v>71</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B24" s="7">
-        <v>46250</v>
+        <v>46247</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="D24" s="5">
-        <v>14764</v>
+        <v>6480</v>
       </c>
       <c r="E24">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B25" s="7">
-        <v>46093</v>
+        <v>46231</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D25" s="5">
-        <v>9432</v>
+        <v>63247</v>
       </c>
       <c r="E25">
-        <v>163</v>
+        <v>25</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B26" s="7">
-        <v>46162</v>
+        <v>46231</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="D26" s="5">
-        <v>10044</v>
+        <v>121984</v>
       </c>
       <c r="E26">
-        <v>94</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B27" s="7">
-        <v>46225</v>
+        <v>45782</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D27" s="5">
-        <v>29612</v>
+        <v>13455</v>
       </c>
       <c r="E27">
-        <v>31</v>
+        <v>474</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="B28" s="7">
-        <v>46247</v>
+        <v>46238</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="D28" s="5">
-        <v>6480</v>
+        <v>3798</v>
       </c>
       <c r="E28">
-        <v>9</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="B29" s="7">
-        <v>46231</v>
+        <v>45511</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="D29" s="5">
-        <v>63247</v>
+        <v>11572</v>
       </c>
       <c r="E29">
-        <v>25</v>
+        <v>745</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="B30" s="7">
-        <v>46231</v>
+        <v>46191</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="D30" s="5">
-        <v>121984</v>
+        <v>31368</v>
       </c>
       <c r="E30">
-        <v>25</v>
+        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="B31" s="7">
-        <v>45782</v>
+        <v>45558</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="D31" s="5">
-        <v>13455</v>
+        <v>20249</v>
       </c>
       <c r="E31">
-        <v>474</v>
+        <v>698</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>184</v>
+        <v>197</v>
       </c>
       <c r="B32" s="7">
-        <v>46238</v>
+        <v>46176</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>185</v>
+        <v>198</v>
       </c>
       <c r="D32" s="5">
-        <v>3798</v>
+        <v>5133</v>
       </c>
       <c r="E32">
-        <v>18</v>
+        <v>80</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>186</v>
+        <v>213</v>
       </c>
       <c r="B33" s="7">
-        <v>46214</v>
+        <v>46250</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>187</v>
+        <v>214</v>
       </c>
       <c r="D33" s="5">
-        <v>7564</v>
+        <v>28138</v>
       </c>
       <c r="E33">
-        <v>42</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>186</v>
+        <v>213</v>
       </c>
       <c r="B34" s="7">
-        <v>46252</v>
+        <v>46250</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>188</v>
+        <v>215</v>
       </c>
       <c r="D34" s="5">
-        <v>15129</v>
+        <v>1480</v>
       </c>
       <c r="E34">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>189</v>
+        <v>228</v>
       </c>
       <c r="B35" s="7">
-        <v>45511</v>
+        <v>45608</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>190</v>
+        <v>229</v>
       </c>
       <c r="D35" s="5">
-        <v>11572</v>
+        <v>6730</v>
       </c>
       <c r="E35">
-        <v>745</v>
+        <v>648</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>191</v>
+        <v>230</v>
       </c>
       <c r="B36" s="7">
-        <v>46191</v>
+        <v>46184</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>192</v>
+        <v>231</v>
       </c>
       <c r="D36" s="5">
-        <v>31368</v>
+        <v>10000</v>
       </c>
       <c r="E36">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>193</v>
+        <v>230</v>
       </c>
       <c r="B37" s="7">
-        <v>45558</v>
+        <v>46227</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>194</v>
+        <v>232</v>
       </c>
       <c r="D37" s="5">
-        <v>20249</v>
+        <v>15000</v>
       </c>
       <c r="E37">
-        <v>698</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>195</v>
-      </c>
-      <c r="B38" s="7">
-        <v>46221</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="D38" s="5">
-        <v>27901</v>
-      </c>
-      <c r="E38">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>197</v>
-      </c>
-      <c r="B39" s="7">
-        <v>46176</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="D39" s="5">
-        <v>5133</v>
-      </c>
-      <c r="E39">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>199</v>
-      </c>
-      <c r="B40" s="7">
-        <v>45727</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="D40" s="5">
-        <v>13824</v>
-      </c>
-      <c r="E40">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>199</v>
-      </c>
-      <c r="B41" s="7">
-        <v>45755</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="D41" s="5">
-        <v>29952</v>
-      </c>
-      <c r="E41">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>199</v>
-      </c>
-      <c r="B42" s="7">
-        <v>45817</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="D42" s="5">
-        <v>16632</v>
-      </c>
-      <c r="E42">
-        <v>439</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>199</v>
-      </c>
-      <c r="B43" s="7">
-        <v>45880</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="D43" s="5">
-        <v>9000</v>
-      </c>
-      <c r="E43">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>199</v>
-      </c>
-      <c r="B44" s="7">
-        <v>45906</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="D44" s="5">
-        <v>22677</v>
-      </c>
-      <c r="E44">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>199</v>
-      </c>
-      <c r="B45" s="7">
-        <v>45911</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D45" s="5">
-        <v>47236</v>
-      </c>
-      <c r="E45">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>199</v>
-      </c>
-      <c r="B46" s="7">
-        <v>45985</v>
-      </c>
-      <c r="C46" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="D46" s="5">
-        <v>5356</v>
-      </c>
-      <c r="E46">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>199</v>
-      </c>
-      <c r="B47" s="7">
-        <v>46058</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="D47" s="5">
-        <v>9619</v>
-      </c>
-      <c r="E47">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>199</v>
-      </c>
-      <c r="B48" s="7">
-        <v>46088</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="D48" s="5">
-        <v>3024</v>
-      </c>
-      <c r="E48">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>199</v>
-      </c>
-      <c r="B49" s="7">
-        <v>46119</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D49" s="5">
-        <v>3024</v>
-      </c>
-      <c r="E49">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>199</v>
-      </c>
-      <c r="B50" s="7">
-        <v>46175</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="D50" s="5">
-        <v>1405</v>
-      </c>
-      <c r="E50">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>199</v>
-      </c>
-      <c r="B51" s="7">
-        <v>46214</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D51" s="5">
-        <v>3240</v>
-      </c>
-      <c r="E51">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>199</v>
-      </c>
-      <c r="B52" s="7">
-        <v>46255</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="D52" s="5">
-        <v>19411</v>
-      </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>213</v>
-      </c>
-      <c r="B53" s="7">
-        <v>46250</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="D53" s="5">
-        <v>28138</v>
-      </c>
-      <c r="E53">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>213</v>
-      </c>
-      <c r="B54" s="7">
-        <v>46250</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="D54" s="5">
-        <v>1480</v>
-      </c>
-      <c r="E54">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>127</v>
-      </c>
-      <c r="B55" s="7">
-        <v>45273</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="D55" s="5">
-        <v>230</v>
-      </c>
-      <c r="E55">
-        <v>983</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>127</v>
-      </c>
-      <c r="B56" s="7">
-        <v>45273</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="D56" s="5">
-        <v>3456</v>
-      </c>
-      <c r="E56">
-        <v>983</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>127</v>
-      </c>
-      <c r="B57" s="7">
-        <v>45299</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="D57" s="5">
-        <v>5760</v>
-      </c>
-      <c r="E57">
-        <v>957</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>127</v>
-      </c>
-      <c r="B58" s="7">
-        <v>45611</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="D58" s="5">
-        <v>1728</v>
-      </c>
-      <c r="E58">
-        <v>645</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>127</v>
-      </c>
-      <c r="B59" s="7">
-        <v>45752</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>220</v>
-      </c>
-      <c r="D59" s="5">
-        <v>20736</v>
-      </c>
-      <c r="E59">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>127</v>
-      </c>
-      <c r="B60" s="7">
-        <v>45903</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="D60" s="5">
-        <v>32880</v>
-      </c>
-      <c r="E60">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>127</v>
-      </c>
-      <c r="B61" s="7">
-        <v>45987</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="D61" s="5">
-        <v>26046</v>
-      </c>
-      <c r="E61">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>127</v>
-      </c>
-      <c r="B62" s="7">
-        <v>46099</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="D62" s="5">
-        <v>38346</v>
-      </c>
-      <c r="E62">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>127</v>
-      </c>
-      <c r="B63" s="7">
-        <v>46122</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>224</v>
-      </c>
-      <c r="D63" s="5">
-        <v>20</v>
-      </c>
-      <c r="E63">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>127</v>
-      </c>
-      <c r="B64" s="7">
-        <v>46244</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>225</v>
-      </c>
-      <c r="D64" s="5">
-        <v>31680</v>
-      </c>
-      <c r="E64">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>127</v>
-      </c>
-      <c r="B65" s="7">
-        <v>46255</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="D65" s="5">
-        <v>12499</v>
-      </c>
-      <c r="E65">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>127</v>
-      </c>
-      <c r="B66" s="7">
-        <v>46255</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="D66" s="5">
-        <v>13608</v>
-      </c>
-      <c r="E66">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>228</v>
-      </c>
-      <c r="B67" s="7">
-        <v>45608</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="D67" s="5">
-        <v>6730</v>
-      </c>
-      <c r="E67">
-        <v>648</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>230</v>
-      </c>
-      <c r="B68" s="7">
-        <v>46184</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="D68" s="5">
-        <v>10000</v>
-      </c>
-      <c r="E68">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>230</v>
-      </c>
-      <c r="B69" s="7">
-        <v>46227</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="D69" s="5">
-        <v>15000</v>
-      </c>
-      <c r="E69">
         <v>29</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E69" xr:uid="{7ECFBB88-5200-475D-B171-1F2F42D2B185}"/>
+  <autoFilter ref="A1:E37" xr:uid="{7ECFBB88-5200-475D-B171-1F2F42D2B185}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C576D64E-905A-4FAB-B026-4747CBD4E42A}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" customWidth="1"/>
@@ -4286,7 +3147,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G17" xr:uid="{C576D64E-905A-4FAB-B026-4747CBD4E42A}"/>
+  <autoFilter ref="A1:E17" xr:uid="{C576D64E-905A-4FAB-B026-4747CBD4E42A}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>